<commit_message>
feat: add explicit vertical layout regions
</commit_message>
<xml_diff>
--- a/scratch/demo_output.xlsx
+++ b/scratch/demo_output.xlsx
@@ -15,6 +15,7 @@
     <sheet name="5 Conditions" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="6 Scalar Types" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="7 Nested Groups" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="8 Region Isolation" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="$#,##0;[Red]-$#,##0;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,6 +105,11 @@
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="FF203040"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="10">
@@ -238,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -347,6 +353,21 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1045,6 +1066,36 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="A17" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Region Isolation</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>3 measured lanes</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>blue band moves</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>gold band stays</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>visually inspect</t>
+        </is>
+      </c>
+    </row>
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
@@ -2243,4 +2294,285 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>Explicit region isolation</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="3" t="n"/>
+    </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>A:J is one shift="cells" region. Its three lanes are measured together; K:P is outside the boundary and must stay fixed.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="40" t="inlineStr">
+        <is>
+          <t>LEFT — 3 items</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>MIDDLE — 5 items</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="40" t="inlineStr">
+        <is>
+          <t>RIGHT — 2 items</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>OUTSIDE REGION</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>A:J REGION BOUNDARY</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Left A</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n"/>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>LEFT</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Middle 1</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="n"/>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>MIDDLE</t>
+        </is>
+      </c>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>Right 1</t>
+        </is>
+      </c>
+      <c r="H6" s="42" t="n"/>
+      <c r="I6" s="42" t="inlineStr">
+        <is>
+          <t>RIGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Left B</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>LEFT</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Middle 2</t>
+        </is>
+      </c>
+      <c r="E7" s="26" t="n"/>
+      <c r="F7" s="26" t="inlineStr">
+        <is>
+          <t>MIDDLE</t>
+        </is>
+      </c>
+      <c r="G7" s="42" t="inlineStr">
+        <is>
+          <t>Right 2</t>
+        </is>
+      </c>
+      <c r="H7" s="42" t="n"/>
+      <c r="I7" s="42" t="inlineStr">
+        <is>
+          <t>RIGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Left C</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>LEFT</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Middle 3</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="n"/>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>MIDDLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Middle 4</t>
+        </is>
+      </c>
+      <c r="E9" s="26" t="n"/>
+      <c r="F9" s="26" t="inlineStr">
+        <is>
+          <t>MIDDLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Middle 5</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>MIDDLE</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>GOLD BAND — outside A:J, stays on row 10</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>BLUE BAND — inside A:J, expected at row 14 after tallest lane adds four rows</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A14:J14"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="K10:P10"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="K4:P4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>